<commit_message>
activity and notification changes
</commit_message>
<xml_diff>
--- a/frontend/public/UM_BU_Template.xlsx
+++ b/frontend/public/UM_BU_Template.xlsx
@@ -1,55 +1,86 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aravi\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45D8559-D836-41FE-AB42-770194F0839C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{08E0AEA7-8564-48AF-AA3B-DBBDFCBF2F35}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="UM_BU Template" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="0"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>UM_BU Template</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>Email Address</t>
-  </si>
-  <si>
-    <t>Mobile Number</t>
-  </si>
-  <si>
-    <t>Employee Type</t>
-  </si>
-  <si>
-    <t>Department</t>
-  </si>
-  <si>
-    <t>Sub Department</t>
-  </si>
-  <si>
-    <t>Level</t>
-  </si>
-  <si>
-    <t>Role Selection</t>
-  </si>
-  <si>
-    <t>Password</t>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Aravinth Raj</dc:creator>
+  <cp:lastModifiedBy>Aravinth Raj</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-13T06:21:18Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-13T12:40:18Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>full_name</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>employee_id</t>
+  </si>
+  <si>
+    <t>role</t>
+  </si>
+  <si>
+    <t>designation</t>
+  </si>
+  <si>
+    <t>level</t>
+  </si>
+  <si>
+    <t>department</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>account_status</t>
+  </si>
+  <si>
+    <t>Aravinth Nagaraj</t>
   </si>
   <si>
     <t>Aravinth</t>
@@ -61,27 +92,33 @@
     <t>aravinth@gmail.com</t>
   </si>
   <si>
-    <t>Quality Control</t>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>ARAV1234</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Quality Staff</t>
+  </si>
+  <si>
+    <t>L2</t>
   </si>
   <si>
     <t>Mixing</t>
   </si>
   <si>
-    <t>L2</t>
-  </si>
-  <si>
-    <t>Quality Staff</t>
-  </si>
-  <si>
-    <t>Dsm@1234</t>
-  </si>
-  <si>
-    <t>ADMIN</t>
+    <t>1992-05-12</t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -637,7 +674,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -932,24 +969,48 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aravi\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45D8559-D836-41FE-AB42-770194F0839C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{08E0AEA7-8564-48AF-AA3B-DBBDFCBF2F35}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="UM_BU Template" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="0"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4562F32C-B9F8-459B-812B-17B5472F90BE}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.109375" customWidth="1"/>
-    <col min="2" max="2" width="11.21875" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.88671875" customWidth="1"/>
-    <col min="5" max="5" width="17.6640625" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" customWidth="1"/>
-    <col min="7" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" customWidth="1"/>
-    <col min="10" max="10" width="19.33203125" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -980,62 +1041,74 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2">
         <v>9876543210</v>
       </c>
-      <c r="E2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="J2" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="K2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J3" s="1"/>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N3" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E278" xr:uid="{94B26BC8-B797-468F-A63A-7FACF0F7252E}">
-      <formula1>"EMP, SUP, ADMIN"</formula1>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H278" xr:uid="{71675C34-5F01-4379-919C-E74E5A6D5352}">
+      <formula1>"Admin, Quality Staff, Manager"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F278" xr:uid="{AD8D28E3-F540-469A-971F-763E19521E7D}">
-      <formula1>"Quality Control, Electrical, Mechincal"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J278" xr:uid="{26EC37F9-C4EE-4654-9637-CFF482FDEBD3}">
+      <formula1>"L1, L2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G278" xr:uid="{93D27A04-EBDE-4CCA-8EFE-82A09421943B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K278" xr:uid="{93D27A04-EBDE-4CCA-8EFE-82A09421943B}">
       <formula1>"Mixing, Blow Room, Carding, Comber, Draw Frame, Simplex, Spinning, Autoconer, Wrapping"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H278" xr:uid="{26EC37F9-C4EE-4654-9637-CFF482FDEBD3}">
-      <formula1>"L1, L2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I278" xr:uid="{71675C34-5F01-4379-919C-E74E5A6D5352}">
-      <formula1>"Quality Staff, Admin, Manager"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Password" error="Password must be at least 8 characters, contain a number, an uppercase letter, a lowercase letter, and a special character (@, #, or $)." sqref="J2:J278" xr:uid="{E8E326CE-28F2-48EC-876A-0CF2B6F961F3}">
-      <formula1>AND(LEN(J2)&gt;=8, COUNT(FIND(ROW(INDIRECT("1:10"))-1, J2))&gt;0, SUMPRODUCT(--ISNUMBER(SEARCH(MID(J2,ROW(INDIRECT("1:"&amp;LEN(J2))),1),"@#$")))&gt;0, NOT(EXACT(LOWER(J2), J2)), NOT(EXACT(UPPER(J2), J2)))</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N278" xr:uid="{AD8D28E3-F540-469A-971F-763E19521E7D}">
+      <formula1>"Active, Inactive"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>